<commit_message>
fix: move headless and slowMo config to playwright.config.ts and clean up test files
</commit_message>
<xml_diff>
--- a/TestData/WorkflowTestingQuestion.xlsx
+++ b/TestData/WorkflowTestingQuestion.xlsx
@@ -412,7 +412,7 @@
         <v>Who is the Finance Minister of India?</v>
       </c>
       <c r="B2" t="str">
-        <v>RELLAB1</v>
+        <v>Response successfully retrieved.</v>
       </c>
     </row>
     <row r="3">
@@ -420,7 +420,7 @@
         <v>Who is the current Chief Election Commissioner (CEC) of India, tasked with overseeing recent state and national electoral processes?</v>
       </c>
       <c r="B3" t="str">
-        <v>RELLAB1</v>
+        <v>Response successfully retrieved.</v>
       </c>
     </row>
     <row r="4">
@@ -428,7 +428,7 @@
         <v>Which unique high-altitude rail bridge—acclaimed as the world's highest railway bridge spanning the Chenab River—was fully operationalised by Indian Railways to provide all-weather connectivity to the Kashmir Valley?</v>
       </c>
       <c r="B4" t="str">
-        <v>RELLAB1</v>
+        <v>Response successfully retrieved.</v>
       </c>
     </row>
     <row r="5">
@@ -436,7 +436,7 @@
         <v>In the field of space exploration, what is the official name of ISRO’s ambitious crewed orbital spacecraft mission, which successfully completed its initial uncrewed test flights ahead of launching Indian astronauts into space?</v>
       </c>
       <c r="B5" t="str">
-        <v>RELLAB1</v>
+        <v>Response successfully retrieved.</v>
       </c>
     </row>
     <row r="6">
@@ -444,7 +444,7 @@
         <v>India's first indigenous solar observation mission, which placed a spacecraft at the Lagrange Point 1 (L1) to study solar winds and coronal mass ejections, is known by what name?</v>
       </c>
       <c r="B6" t="str">
-        <v>RELLAB1</v>
+        <v>Response successfully retrieved.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>